<commit_message>
Publish the companion site
</commit_message>
<xml_diff>
--- a/files/family_decomposition.xlsx
+++ b/files/family_decomposition.xlsx
@@ -698,7 +698,7 @@
     <row r="8" ht="171" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Note. Two parallel Mundlak mixed-effects models on the MIDUS M2MR2 twin/sibling subsample: (i) cross-sectional at W1 (Y_w1 on B/W-partitioned focal X + age_W1 B/W + sex + pair random intercept) and (ii) 9-year change (Y_w2 on the same partition plus the autoregressive B/W-partitioned Y_w1 and age_W2). Focal predictors differ by analysis: CS uses the top-20-∩-stable variables (top20_stability ≥ 0.60) from cs1_cross_sectional bootstrap SHAP; change uses the stable A4 longitudinal SHAP set, excluding the autoregressive W1 outcome. All_paired = MZ + DZ_SS + DZ_OS + non-twin siblings (primary); MZ_sens = MZ pairs only (sensitivity). ICC_MZ is the outcome null-model intraclass correlation (σ²_u / (σ²_u + σ²_e)); overview denominators are domain-level ICC counts, while coefficient rows carry predictor-complete n_pairs and n_MZ. Allostatic-load rows use the AL_noAnthro biomarker sample and should not be assumed to share frailty/cognition denominators. CS stratum is consistently higher than change across domains, motivating the CS analysis as the primary within-family test. "FDR-surviving β_W" = predictors with Benjamini–Hochberg q ≤ 0.05 within each (analysis × group × outcome) predictor set. Following Turkheimer (2000) and Harden (2021), β_W indexes familial resemblance of psychosocial–aging coupling net of shared background, not heritability of the trait. Full predictor-level results appear in the "CS full", "Change full", and "FDR-surviving β_W" sheets; methods detail in "Notes".</t>
+          <t>Note. Two parallel Mundlak mixed-effects models on the MIDUS 2 and MIDUS Refresher twin subsample: (i) cross-sectional at W1 (Y_w1 on B/W-partitioned focal X + age_W1 B/W + sex + pair random intercept) and (ii) 9-year change (Y_w2 on the same partition plus the autoregressive B/W-partitioned Y_w1 and age_W2). Focal predictors differ by analysis: CS uses the top-20-∩-stable variables (top20_stability ≥ 0.60) from cs1_cross_sectional bootstrap SHAP; change uses the stable A4 longitudinal SHAP set, excluding the autoregressive W1 outcome. All_paired = MZ + DZ_SS + DZ_OS twin pairs (primary); MZ_sens = MZ pairs only (sensitivity). ICC_MZ is the outcome null-model intraclass correlation (σ²_u / (σ²_u + σ²_e)); overview denominators are domain-level ICC counts, while coefficient rows carry predictor-complete n_pairs and n_MZ. Allostatic-load rows use the allostatic-load biomarker sample and should not be assumed to share frailty/cognition denominators. CS stratum is consistently higher than change across domains, motivating the CS analysis as the primary within-family test. "FDR-surviving β_W" = predictors with Benjamini–Hochberg q ≤ 0.05 within each (analysis × group × outcome) predictor set. Following Turkheimer (2000) and Harden (2021), β_W indexes familial resemblance of psychosocial–aging coupling net of shared background, not heritability of the trait. Full predictor-level results appear in the "CS full", "Change full", and "FDR-surviving β_W" sheets; methods detail in "Notes".</t>
         </is>
       </c>
     </row>
@@ -1055,10 +1055,10 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="156" customHeight="1">
+    <row r="14" ht="126" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Note. Null-model intraclass correlations (ICC = σ²_u / (σ²_u + σ²_e)) from mixed-effects regressions with pair random intercept and age (decomposed B/W) + sex fixed covariates. CS column: ICC of the Wave-1 outcome only (no lagged Y). Change column: ICC of the Wave-2 outcome after conditioning on Wave-1 outcome (B/W-partitioned); this is the familial resemblance of the residual change, not of raw W2 state. Sibling strata: MZ (monozygotic), DZ_SS (dizygotic same-sex), All_paired (MZ + DZ_SS + DZ_OS + non-twin siblings). CS n_pairs exceeds change n_pairs because the change model additionally requires W2 outcome presence. Cross-domain ordering differs between columns: at W1, cognition (.62) &gt; AL (.44) &gt; frailty (.37); for change, AL (.42) &gt; cognition (.32) &gt; frailty (.18).</t>
+          <t>Note. Null-model intraclass correlations (ICC = σ²_u / (σ²_u + σ²_e)) from mixed-effects regressions with pair random intercept and age (decomposed B/W) + sex fixed covariates. CS column: ICC of the Wave-1 outcome only (no lagged Y). Change column: ICC of the Wave-2 outcome after conditioning on Wave-1 outcome (B/W-partitioned); this is the familial resemblance of the residual change, not of raw W2 state. Sibling strata: MZ (monozygotic), DZ_SS (dizygotic same-sex), All_paired (MZ + DZ_SS + DZ_OS). CS n_pairs exceeds change n_pairs because the change model additionally requires W2 outcome presence.</t>
         </is>
       </c>
     </row>
@@ -2694,10 +2694,10 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="126" customHeight="1">
+    <row r="34" ht="96" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Note. All within-family (β_W) predictors with Benjamini–Hochberg q ≤ 0.05, pooled across analyses. Analysis: cs = cross-sectional W1; change = W1→W2 with autoregressive W1 control. Group: All_paired = primary; MZ_sensitivity = MZ-only robustness check. β_W raw = unstandardized coefficient; β_W std = Snijders–Bosker level-specific standardized; 95% CI from 1000× pairs-level bootstrap. n_pairs is predictor-complete for the displayed group; n_MZ is the matched predictor-complete MZ denominator for the same coefficient where available, with n_MZ_status marking skipped MZ models. q-values are BH-FDR across all predictors within each (analysis × group × outcome) table. 26 rows total (n by analysis-group: CS All_paired = 17, CS MZ_sens = 8, change All_paired = 1, change MZ_sens = 0) — CS carries 25 of the 26 FDR-surviving within-family signals; 9-year change is essentially empty at current sibling power except for blue-collar occupation → cognitive decline. Between-family (β_B) coefficients for the same variable–outcome pairs are in the "CS full" / "Change full" sheets.</t>
+          <t>Note. All within-family (β_W) predictors with Benjamini–Hochberg q ≤ 0.05, pooled across analyses. Analysis: cs = cross-sectional W1; change = W1→W2 with autoregressive W1 control. Group: All_paired = primary; MZ_sensitivity = MZ-only robustness check. β_W raw = unstandardized coefficient; β_W std = Snijders–Bosker level-specific standardized; 95% CI from 1000× pairs-level bootstrap. n_pairs is predictor-complete for the displayed group; n_MZ is the matched predictor-complete MZ denominator for the same coefficient where available, with n_MZ_status marking skipped MZ models. q-values are BH-FDR across all predictors within each (analysis × group × outcome) table. Between-family (β_B) coefficients for the same variable–outcome pairs are in the "CS full" / "Change full" sheets.</t>
         </is>
       </c>
     </row>
@@ -10037,7 +10037,7 @@
     <row r="101" ht="81" customHeight="1">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>Note. Full cross-sectional (W1) within/between-family decomposition. Each row: one focal predictor × group × outcome. Model: Y_w1 = β_B · X̄_j + β_W · (X_ij − X̄_j) + age_W1 (B/W) + sex + (1|pair_id). β_W = within-family effect; β_B = between-family effect; β_W/β_B = attenuation ratio (reported when |β_B| &gt; 0.5·SE(β_B)). Standardized β use Snijders–Bosker (2012) level-specific SDs. CI from 1000× pairs-level bootstrap. q-values are BH-FDR within each (group × outcome) table; ✓ in the final column flags q ≤ 0.05. n_pairs and n_MZ are predictor-complete coefficient-row denominators; n_MZ_status marks variables not fitted in the MZ sensitivity after discordance/power filters. Table S4/Overview uses domain-level ICC denominators. Focal set: top-20 mean|SHAP| ∩ stable (top20_stability ≥ 0.60) from cs1_cross_sectional bootstrap SHAP per outcome (15/20/11 predictors for frailty/cognition/AL after pair-level filters). Categorical dummies (workStatus, occGroup, workIndustry) are dropped when they have &lt;15 discordant pairs within-group.</t>
+          <t>Note. Full cross-sectional (W1) within/between-family decomposition. Each row: one focal predictor × group × outcome. Model: Y_w1 = β_B · X̄_j + β_W · (X_ij − X̄_j) + age_W1 (B/W) + sex + (1|pair_id). β_W = within-family effect; β_B = between-family effect; β_W/β_B = attenuation ratio (reported when |β_B| &gt; 0.5·SE(β_B)). Standardized β use Snijders–Bosker (2012) level-specific SDs. CI from 1000× pairs-level bootstrap. q-values are BH-FDR within each (group × outcome) table; ✓ in the final column flags q ≤ 0.05. n_pairs and n_MZ are predictor-complete coefficient-row denominators; n_MZ_status marks variables not fitted in the MZ sensitivity after discordance/power filters. Table S4/Overview uses domain-level ICC denominators. Focal set: top-20 mean|SHAP| ∩ stable (top20_stability ≥ 0.60) from cs1_cross_sectional bootstrap SHAP per outcome, after pair-level filters. Categorical dummies (workStatus, occGroup, workIndustry) are estimated when at least two pairs are discordant within-group.</t>
         </is>
       </c>
     </row>
@@ -15432,10 +15432,10 @@
       </c>
       <c r="P74" s="3" t="inlineStr"/>
     </row>
-    <row r="76" ht="81" customHeight="1">
+    <row r="76" ht="66" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>Note. Full 9-year change (W1 → W2) within/between-family decomposition. Model: Y_w2 = β_B · X̄_j + β_W · (X_ij − X̄_j) + α_B · Ȳ_w1,j + α_W · (Y_w1,ij − Ȳ_w1,j) + age_W2 (B/W) + sex + (1|pair_id). The autoregressive Y_w1 terms absorb baseline state, so β_W reports within-pair predictor effect on residual 9-year change. Standardized β: Snijders–Bosker level-specific. CI from 1000× pairs-level bootstrap. q-values are BH-FDR within each (group × outcome) table; ✓ flags q ≤ 0.05. Focal set: stable A4 longitudinal bootstrap SHAP per outcome, excluding the autoregressive W1 outcome. Sample sizes are roughly half the CS sizes because complete W1+W2 outcome data are required; only one predictor (blue-collar occupation → cognition, All_paired q = 0.001) survives FDR at this power. n_pairs and n_MZ are predictor-complete coefficient-row denominators; n_MZ_status marks variables not fitted in the MZ sensitivity after discordance/power filters. Table S4/Overview uses domain-level ICC denominators.</t>
+          <t>Note. Full 9-year change (W1 → W2) within/between-family decomposition. Model: Y_w2 = β_B · X̄_j + β_W · (X_ij − X̄_j) + α_B · Ȳ_w1,j + α_W · (Y_w1,ij − Ȳ_w1,j) + age_W2 (B/W) + sex + (1|pair_id). The autoregressive Y_w1 terms absorb baseline state, so β_W reports within-pair predictor effect on residual 9-year change. Standardized β: Snijders–Bosker level-specific. CI from 1000× pairs-level bootstrap. q-values are BH-FDR within each (group × outcome) table; ✓ flags q ≤ 0.05. Focal set: stable A4 longitudinal bootstrap SHAP per outcome, excluding the autoregressive W1 outcome. Sample sizes are roughly half the CS sizes because complete W1+W2 outcome data are required. n_pairs and n_MZ are predictor-complete coefficient-row denominators; n_MZ_status marks variables not fitted in the MZ sensitivity after discordance/power filters. Table S4/Overview uses domain-level ICC denominators.</t>
         </is>
       </c>
     </row>
@@ -15472,7 +15472,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Two parallel Mundlak models fit on twin/sibling pairs from MIDUS 2 Refresher + MIDUS 3 (M2MR2) sibling/twin subsample:</t>
+          <t>Two parallel Mundlak models fit on twin pairs from MIDUS 2 and the MIDUS Refresher (Wave 1), followed at MIDUS 3 and Refresher 2 (Wave 2):</t>
         </is>
       </c>
     </row>
@@ -15554,7 +15554,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Primary model: All_paired (MZ + DZ_SS + DZ_OS + non-twin siblings).</t>
+          <t>Primary model: All_paired (MZ + DZ_SS + DZ_OS twin pairs).</t>
         </is>
       </c>
     </row>
@@ -15575,14 +15575,14 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Allostatic-load sibling rows use AL_noAnthro biomarker-specific sample counts because the AL biomarker longitudinal sample keeps the sibling-exclusion exception for power.</t>
+          <t>Allostatic-load sibling rows use allostatic-load biomarker-specific sample counts because the AL biomarker longitudinal sample keeps the sibling-exclusion exception for power.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Categorical variables (workStatus, occGroup, workIndustry) are expanded to k-1 dummies with substantive groupings; dummies with &lt;15 discordant pairs are excluded.</t>
+          <t>Categorical variables (workStatus, occGroup, workIndustry) are expanded to k-1 dummies with substantive groupings; dummies with fewer than two discordant pairs are excluded.</t>
         </is>
       </c>
     </row>
@@ -15599,7 +15599,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Outcome null-model ICC_MZ by zygosity: CS stratum is substantially higher than the change stratum for cognition and frailty (concurrent state carries more heritable signal than its 9-year change).</t>
+          <t>Outcome null-model ICC_MZ by zygosity: higher cross-sectionally than for 9-year change in all three outcomes.</t>
         </is>
       </c>
     </row>

</xml_diff>